<commit_message>
update some bugs on saved array dimension -> audio stimuli and its features are saved as (time, feature, speaker,), if envelope or raw audio, featur=1, but dim is retained
</commit_message>
<xml_diff>
--- a/recently_presented_datasets.xlsx
+++ b/recently_presented_datasets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sean\Documents\Seafile\ZYMdeDocument\24-12-SuperPrepare\SuperPrepare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2292C296-AFCE-47AF-A1E4-26EF669058FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6B98E1-7EDD-49DD-A59F-BD2653518F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7538" yWindow="-75" windowWidth="21337" windowHeight="15135" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>https://www.sciencedirect.com/science/article/pii/S1053811919308742#:~:text=Position%20of%20attended%20moving%20sound%20can%20be%20decoded,stimulus%20trajectory%20was%20weakly%20tracked%20by%20delta%20EEG.</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>缺少标签和真实位置的对应</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/9997944</t>
   </si>
 </sst>
 </file>
@@ -403,6 +406,11 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+    </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>5</v>

</xml_diff>